<commit_message>
chore: update Instagram report 2026-09-14 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-13 06:44:52</t>
+          <t>取得日時：2026-09-14 05:53:52</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-12</t>
+          <t>比較基準：2026-09-13</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>344</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12T12:10:07+0000</t>
+          <t>2026-09-13T15:26:30+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -939,17 +939,17 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>106</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1095,17 +1095,17 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1147,17 +1147,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>554</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>555</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1547</t>
+          <t>1548</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1251,17 +1251,17 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>346</t>
+          <t>347</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>86</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12T05:40:05+0000</t>
+          <t>2026-09-13T09:18:09+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1405,19 +1405,19 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1506,37 +1506,37 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T12:31:05+0000</t>
+          <t>2026-09-13T11:17:34+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1558,37 +1558,37 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>172</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>174</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29T11:07:12+0000</t>
+          <t>2026-09-13T12:45:57+0000</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-15 05:57
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-14 06:44:42</t>
+          <t>取得日時：2026-09-15 05:57:08</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-13</t>
+          <t>比較基準：2026-09-14</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>344</t>
+          <t>347</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13T15:26:30+0000</t>
+          <t>2026-09-14T15:59:53+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -937,7 +937,7 @@
           <t>33</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -947,9 +947,9 @@
           <t>106</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1093,7 +1093,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1103,9 +1103,9 @@
           <t>21</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1152,12 +1152,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>555</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1548</t>
+          <t>1549</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>348</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,9 +1301,9 @@
           <t>86</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+3件</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,9 +1311,9 @@
           <t>233</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,24 +1363,24 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09T22:57:15+0000</t>
+          <t>2026-09-13T23:28:38+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1402,37 +1402,37 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07T12:41:19+0000</t>
+          <t>2026-09-14T00:07:42+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1506,17 +1506,17 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>93</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13T11:17:34+0000</t>
+          <t>2026-09-14T01:50:40+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1561,9 +1561,9 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1571,9 +1571,9 @@
           <t>174</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-16 05:55
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-15 06:47:16</t>
+          <t>取得日時：2026-09-16 05:55:04</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-14</t>
+          <t>比較基準：2026-09-15</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>350</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14T15:59:53+0000</t>
+          <t>2026-09-15T12:10:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,19 +729,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1142,32 +1142,32 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12T15:25:04+0000</t>
+          <t>2026-09-15T14:46:53+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1549</t>
+          <t>1550</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,7 +1249,7 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1259,9 +1259,9 @@
           <t>348</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,9 +1353,9 @@
           <t>33</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,7 +1363,7 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1405,9 +1405,9 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,9 +1415,9 @@
           <t>51</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,9 +1509,9 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1519,9 +1519,9 @@
           <t>93</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-17 05:56
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-16 06:45:18</t>
+          <t>取得日時：2026-09-17 05:56:01</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-15</t>
+          <t>比較基準：2026-09-16</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>353</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15T12:10:06+0000</t>
+          <t>2026-09-16T12:10:07+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>25</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,24 +947,24 @@
           <t>106</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12T10:15:02+0000</t>
+          <t>2026-09-16T10:20:01+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,24 +1103,24 @@
           <t>21</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12T13:30:22+0000</t>
+          <t>2026-09-16T11:02:11+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15T14:46:53+0000</t>
+          <t>2026-09-16T10:56:55+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>555</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1550</t>
+          <t>1551</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,19 +1249,19 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>348</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,19 +1311,19 @@
           <t>233</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13T09:18:09+0000</t>
+          <t>2026-09-16T09:45:40+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-18 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-17 06:46:54</t>
+          <t>取得日時：2026-09-18 05:53:48</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-16</t>
+          <t>比較基準：2026-09-17</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>356</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16T12:10:07+0000</t>
+          <t>2026-09-17T12:10:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16T10:20:01+0000</t>
+          <t>2026-09-17T10:20:01+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16T11:02:11+0000</t>
+          <t>2026-09-17T11:48:03+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16T10:56:55+0000</t>
+          <t>2026-09-17T14:32:54+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>554</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>-1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1551</t>
+          <t>1552</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,7 +1249,7 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1259,9 +1259,9 @@
           <t>347</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>-1人</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,9 +1301,9 @@
           <t>88</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,7 +1311,7 @@
           <t>233</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1427,12 +1427,12 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-19 07:52
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-18 06:44:10</t>
+          <t>取得日時：2026-09-19 07:52:11</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-17</t>
+          <t>比較基準：2026-09-18</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>359</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17T12:10:06+0000</t>
+          <t>2026-09-17T21:46:00+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -937,9 +937,9 @@
           <t>35</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
           <t>106</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17T11:48:03+0000</t>
+          <t>2026-09-18T13:49:30+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17T14:32:54+0000</t>
+          <t>2026-09-18T12:56:42+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1552</t>
+          <t>1553</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,19 +1301,19 @@
           <t>88</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>233</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>94</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-20 07:32
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-19 08:34:35</t>
+          <t>取得日時：2026-09-20 07:32:14</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-18</t>
+          <t>比較基準：2026-09-19</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>362</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,22 +684,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>538</t>
+          <t>539</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17T21:46:00+0000</t>
+          <t>2026-09-19T12:30:01+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,19 +947,19 @@
           <t>106</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17T10:20:01+0000</t>
+          <t>2026-09-19T10:30:02+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18T13:49:30+0000</t>
+          <t>2026-09-19T11:41:15+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18T12:56:42+0000</t>
+          <t>2026-09-19T11:42:46+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1553</t>
+          <t>1554</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
           <t>88</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1311,9 +1311,9 @@
           <t>234</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,24 +1363,24 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13T23:28:38+0000</t>
+          <t>2026-09-19T05:26:13+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>94</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>174</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-21 07:44
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-20 08:29:19</t>
+          <t>取得日時：2026-09-21 07:44:32</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-19</t>
+          <t>比較基準：2026-09-20</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>365</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>539</t>
+          <t>540</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19T12:30:01+0000</t>
+          <t>2026-09-20T12:00:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -937,9 +937,9 @@
           <t>36</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
           <t>106</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1093,9 +1093,9 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,7 +1103,7 @@
           <t>21</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1147,17 +1147,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1554</t>
+          <t>1555</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,19 +1301,19 @@
           <t>88</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>234</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,9 +1353,9 @@
           <t>34</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,7 +1363,7 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>95</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>176</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-22 08:41
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-21 08:29:06</t>
+          <t>取得日時：2026-09-22 08:41:43</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-20</t>
+          <t>比較基準：2026-09-21</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>368</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+4件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>539</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-20T23:15:25+0000</t>
+          <t>2026-09-21T09:30:05+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1093,19 +1093,19 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>56</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1555</t>
+          <t>1556</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,7 +1301,7 @@
           <t>88</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1311,9 +1311,9 @@
           <t>235</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,19 +1353,19 @@
           <t>34</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-23 08:18
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-22 09:16:41</t>
+          <t>取得日時：2026-09-23 08:18:42</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-21</t>
+          <t>比較基準：2026-09-22</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>372</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+4件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>539</t>
+          <t>540</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21T09:30:05+0000</t>
+          <t>2026-09-22T23:10:10+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19T11:41:15+0000</t>
+          <t>2026-09-22T10:25:04+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1556</t>
+          <t>1557</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
           <t>34</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1363,9 +1363,9 @@
           <t>85</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1402,12 +1402,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,24 +1415,24 @@
           <t>51</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14T00:07:42+0000</t>
+          <t>2026-09-22T13:10:46+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-24 08:12
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-23 08:47:51</t>
+          <t>取得日時：2026-09-24 08:12:48</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-22</t>
+          <t>比較基準：2026-09-23</t>
         </is>
       </c>
     </row>
@@ -674,17 +674,17 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>374</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+4件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>541</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22T23:10:10+0000</t>
+          <t>2026-09-23T10:00:02+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -934,37 +934,37 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>106</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19T10:30:02+0000</t>
+          <t>2026-09-23T10:10:02+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1093,9 +1093,9 @@
           <t>15</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,7 +1103,7 @@
           <t>22</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1152,12 +1152,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>59</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>554</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>555</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1557</t>
+          <t>1558</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,24 +1311,24 @@
           <t>235</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16T09:45:40+0000</t>
+          <t>2026-09-23T09:23:32+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1353,19 +1353,19 @@
           <t>34</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1405,9 +1405,9 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,7 +1415,7 @@
           <t>51</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>177</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-25 08:31
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-24 08:56:35</t>
+          <t>取得日時：2026-09-25 08:31:23</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-23</t>
+          <t>比較基準：2026-09-24</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>374</t>
+          <t>377</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T10:00:02+0000</t>
+          <t>2026-09-24T10:30:00+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -937,9 +937,9 @@
           <t>37</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,9 +947,9 @@
           <t>108</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,19 +1103,19 @@
           <t>22</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22T10:25:04+0000</t>
+          <t>2026-09-24T10:27:36+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,12 +1142,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1157,22 +1157,22 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19T11:42:46+0000</t>
+          <t>2026-09-24T14:17:54+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>555</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1558</t>
+          <t>1559</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,9 +1301,9 @@
           <t>91</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+3件</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,7 +1311,7 @@
           <t>235</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
           <t>34</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1363,9 +1363,9 @@
           <t>86</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>177</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-26 08:37
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-25 08:59:57</t>
+          <t>取得日時：2026-09-26 08:37:24</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-24</t>
+          <t>比較基準：2026-09-25</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>380</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24T10:30:00+0000</t>
+          <t>2026-09-25T10:00:04+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24T10:27:36+0000</t>
+          <t>2026-09-25T10:07:45+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>60</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24T14:17:54+0000</t>
+          <t>2026-09-25T13:13:09+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1559</t>
+          <t>1560</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,19 +1249,19 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>347</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,32 +1298,32 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>235</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T09:23:32+0000</t>
+          <t>2026-09-25T09:18:24+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1506,17 +1506,17 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>97</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1526,17 +1526,17 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14T01:50:40+0000</t>
+          <t>2026-09-25T12:29:23+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-27 08:12
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-26 09:08:40</t>
+          <t>取得日時：2026-09-27 08:12:09</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-25</t>
+          <t>比較基準：2026-09-26</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>383</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25T10:00:04+0000</t>
+          <t>2026-09-26T12:00:10+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25T10:07:45+0000</t>
+          <t>2026-09-26T11:19:08+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25T13:13:09+0000</t>
+          <t>2026-09-26T12:18:25+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>555</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1560</t>
+          <t>1561</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,7 +1249,7 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1259,9 +1259,9 @@
           <t>348</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>95</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25T09:18:24+0000</t>
+          <t>2026-09-26T06:40:07+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,24 +1363,24 @@
           <t>86</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19T05:26:13+0000</t>
+          <t>2026-09-26T21:33:22+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,9 +1509,9 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1519,9 +1519,9 @@
           <t>97</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-28 08:27
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-27 08:51:49</t>
+          <t>取得日時：2026-09-28 08:27:02</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-26</t>
+          <t>比較基準：2026-09-27</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>387</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+4件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>542</t>
+          <t>541</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-26T12:00:10+0000</t>
+          <t>2026-09-27T22:45:58+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,24 +947,24 @@
           <t>108</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T10:10:02+0000</t>
+          <t>2026-09-27T10:00:02+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1093,9 +1093,9 @@
           <t>18</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,7 +1103,7 @@
           <t>22</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1147,17 +1147,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>61</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>554</t>
+          <t>555</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1561</t>
+          <t>1562</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,19 +1249,19 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>348</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>97</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-26T06:40:07+0000</t>
+          <t>2026-09-27T06:35:07+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1355,17 +1355,17 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>87</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>177</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>-2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-29 09:36
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-28 08:57:00</t>
+          <t>取得日時：2026-09-29 09:36:49</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-27</t>
+          <t>比較基準：2026-09-28</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>387</t>
+          <t>390</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+4件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-27T22:45:58+0000</t>
+          <t>2026-09-28T22:45:35+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -937,9 +937,9 @@
           <t>38</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
           <t>108</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>555</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1562</t>
+          <t>1563</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>348</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>237</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-26T21:33:22+0000</t>
+          <t>2026-09-28T23:30:05+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>175</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>-2人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-30 08:59
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-29 10:14:28</t>
+          <t>取得日時：2026-09-30 08:59:44</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-28</t>
+          <t>比較基準：2026-09-29</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>392</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28T22:45:35+0000</t>
+          <t>2026-09-29T12:30:02+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,19 +1103,19 @@
           <t>22</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-26T11:19:08+0000</t>
+          <t>2026-09-29T10:51:09+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,12 +1142,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1157,17 +1157,17 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-26T12:18:25+0000</t>
+          <t>2026-09-29T10:32:16+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1563</t>
+          <t>1564</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>348</t>
+          <t>347</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,7 +1301,7 @@
           <t>97</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1311,9 +1311,9 @@
           <t>237</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1355,17 +1355,17 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-01 09:13
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-30 09:45:39</t>
+          <t>取得日時：2026-10-01 09:13:21</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-29</t>
+          <t>比較基準：2026-09-30</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>392</t>
+          <t>396</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+4件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29T12:30:02+0000</t>
+          <t>2026-09-30T22:25:47+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29T10:51:09+0000</t>
+          <t>2026-09-30T10:59:58+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29T10:32:16+0000</t>
+          <t>2026-09-30T09:57:32+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1564</t>
+          <t>1565</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>347</t>
+          <t>348</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
           <t>36</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1363,9 +1363,9 @@
           <t>88</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-02 09:16
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-01 09:49:26</t>
+          <t>取得日時：2026-10-02 09:16:44</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-30</t>
+          <t>比較基準：2026-10-01</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>396</t>
+          <t>399</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+4件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>540</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30T22:25:47+0000</t>
+          <t>2026-10-01T22:11:12+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,37 +726,37 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+0人</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01T14:32:23+0000</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -934,12 +934,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,24 +947,24 @@
           <t>108</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-27T10:00:02+0000</t>
+          <t>2026-10-01T10:00:01+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30T10:59:58+0000</t>
+          <t>2026-10-01T10:32:58+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>63</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30T09:57:32+0000</t>
+          <t>2026-10-01T10:33:45+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1565</t>
+          <t>1566</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,7 +1249,7 @@
           <t>58</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1259,9 +1259,9 @@
           <t>348</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1350,32 +1350,32 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28T23:30:05+0000</t>
+          <t>2026-10-01T22:43:49+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>97</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>175</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-03 09:01
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-02 10:04:56</t>
+          <t>取得日時：2026-10-03 09:01:54</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-01</t>
+          <t>比較基準：2026-10-02</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>402</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01T22:11:12+0000</t>
+          <t>2026-10-02T22:25:08+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -736,17 +736,17 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>40</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+15人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01T14:32:23+0000</t>
+          <t>2026-10-02T14:19:29+0000</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -939,17 +939,17 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>109</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01T10:32:58+0000</t>
+          <t>2026-10-02T10:40:55+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01T10:33:45+0000</t>
+          <t>2026-10-02T10:41:22+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>555</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>556</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1566</t>
+          <t>1567</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,37 +1298,37 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>97</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>237</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-27T06:35:07+0000</t>
+          <t>2026-10-02T05:49:25+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1353,9 +1353,9 @@
           <t>37</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,9 +1363,9 @@
           <t>89</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>177</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-04 08:21
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-03 09:43:26</t>
+          <t>取得日時：2026-10-04 08:21:55</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-02</t>
+          <t>比較基準：2026-10-03</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>405</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02T22:25:08+0000</t>
+          <t>2026-10-03T22:30:35+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -736,17 +736,17 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+15人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02T14:19:29+0000</t>
+          <t>2026-10-03T14:14:53+0000</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -937,7 +937,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -947,9 +947,9 @@
           <t>109</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02T10:40:55+0000</t>
+          <t>2026-10-03T11:54:04+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02T10:41:22+0000</t>
+          <t>2026-10-03T15:34:17+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>556</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1567</t>
+          <t>1568</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02T05:49:25+0000</t>
+          <t>2026-10-03T05:40:05+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,19 +1363,19 @@
           <t>89</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01T22:43:49+0000</t>
+          <t>2026-10-03T07:13:42+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1506,12 +1506,12 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1521,22 +1521,22 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25T12:29:23+0000</t>
+          <t>2026-10-03T13:08:02+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>177</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-05 08:38
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-04 09:01:40</t>
+          <t>取得日時：2026-10-05 08:38:31</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-03</t>
+          <t>比較基準：2026-10-04</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>407</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T22:30:35+0000</t>
+          <t>2026-10-04T09:30:02+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,9 +729,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -739,9 +739,9 @@
           <t>42</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1093,9 +1093,9 @@
           <t>23</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,7 +1103,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1147,17 +1147,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>65</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1568</t>
+          <t>1569</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>102</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1308,17 +1308,17 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>-2人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T05:40:05+0000</t>
+          <t>2026-10-04T05:45:04+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1353,9 +1353,9 @@
           <t>38</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,7 +1363,7 @@
           <t>89</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1511,17 +1511,17 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>177</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-06 10:31
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-05 09:08:48</t>
+          <t>取得日時：2026-10-06 10:31:26</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-04</t>
+          <t>比較基準：2026-10-05</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>411</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>541</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T23:40:29+0000</t>
+          <t>2026-10-05T22:34:47+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,19 +729,19 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+5人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1093,19 +1093,19 @@
           <t>23</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1155,9 +1155,9 @@
           <t>65</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1569</t>
+          <t>1570</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,9 +1301,9 @@
           <t>102</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,9 +1311,9 @@
           <t>236</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>-2人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>100</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>176</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>-1人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-07 09:11
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-06 10:52:52</t>
+          <t>取得日時：2026-10-07 09:11:43</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-05</t>
+          <t>比較基準：2026-10-06</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>414</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>540</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05T22:34:47+0000</t>
+          <t>2026-10-06T22:15:48+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>50</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+5人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T11:54:04+0000</t>
+          <t>2026-10-06T12:38:46+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,12 +1142,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1155,19 +1155,19 @@
           <t>65</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T15:34:17+0000</t>
+          <t>2026-10-06T14:18:16+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1570</t>
+          <t>1571</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,19 +1301,19 @@
           <t>102</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>236</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-08 09:26
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-07 10:00:54</t>
+          <t>取得日時：2026-10-08 09:26:53</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-06</t>
+          <t>比較基準：2026-10-07</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>417</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>539</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06T22:15:48+0000</t>
+          <t>2026-10-07T22:00:10+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,37 +726,37 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+4人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T14:14:53+0000</t>
+          <t>2026-10-07T13:22:54+0000</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1095,17 +1095,17 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06T14:18:16+0000</t>
+          <t>2026-10-07T11:25:33+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1571</t>
+          <t>1572</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>103</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1313,17 +1313,17 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-04T05:45:04+0000</t>
+          <t>2026-10-07T08:53:09+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,24 +1363,24 @@
           <t>89</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T07:13:42+0000</t>
+          <t>2026-10-07T02:18:22+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-09 09:42
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-08 10:16:40</t>
+          <t>取得日時：2026-10-09 09:42:39</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-07</t>
+          <t>比較基準：2026-10-08</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>417</t>
+          <t>420</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07T22:00:10+0000</t>
+          <t>2026-10-08T22:30:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07T13:22:54+0000</t>
+          <t>2026-10-08T15:37:50+0000</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
           <t>24</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1103,9 +1103,9 @@
           <t>27</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07T11:25:33+0000</t>
+          <t>2026-10-08T13:26:06+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1572</t>
+          <t>1573</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,9 +1301,9 @@
           <t>103</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,7 +1311,7 @@
           <t>238</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,9 +1353,9 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,7 +1363,7 @@
           <t>89</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>101</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-10 09:21
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-09 10:24:43</t>
+          <t>取得日時：2026-10-10 09:21:25</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-08</t>
+          <t>比較基準：2026-10-09</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>423</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08T22:30:06+0000</t>
+          <t>2026-10-09T22:30:10+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -731,12 +731,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,19 +1103,19 @@
           <t>27</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06T12:38:46+0000</t>
+          <t>2026-10-09T10:28:47+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08T13:26:06+0000</t>
+          <t>2026-10-09T10:04:32+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1573</t>
+          <t>1574</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-11 08:54
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-10 10:12:43</t>
+          <t>取得日時：2026-10-11 08:54:03</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-09</t>
+          <t>比較基準：2026-10-10</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>423</t>
+          <t>426</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T22:30:10+0000</t>
+          <t>2026-10-10T22:30:07+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,12 +726,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08T15:37:50+0000</t>
+          <t>2026-10-10T15:30:17+0000</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T10:28:47+0000</t>
+          <t>2026-10-10T13:01:36+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09T10:04:32+0000</t>
+          <t>2026-10-10T13:52:12+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1574</t>
+          <t>1575</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,32 +1298,32 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>103</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>238</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07T08:53:09+0000</t>
+          <t>2026-10-10T08:48:13+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,19 +1353,19 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-12 09:02
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-11 09:26:04</t>
+          <t>取得日時：2026-10-12 09:02:01</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-10</t>
+          <t>比較基準：2026-10-11</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>426</t>
+          <t>429</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>539</t>
+          <t>541</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10T22:30:07+0000</t>
+          <t>2026-10-11T22:30:30+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>66</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+12人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1095,17 +1095,17 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1145,9 +1145,9 @@
           <t>28</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1155,7 +1155,7 @@
           <t>67</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>556</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>557</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1575</t>
+          <t>1576</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>107</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10T08:48:13+0000</t>
+          <t>2026-10-11T06:05:06+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1363,9 +1363,9 @@
           <t>90</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>102</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>13</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-13 11:17
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-12 09:44:04</t>
+          <t>取得日時：2026-10-13 11:17:09</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-11</t>
+          <t>比較基準：2026-10-12</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>429</t>
+          <t>432</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11T22:30:30+0000</t>
+          <t>2026-10-12T22:30:05+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+12人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1093,7 +1093,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1103,9 +1103,9 @@
           <t>30</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>+3人</t>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1145,19 +1145,19 @@
           <t>28</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>557</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1576</t>
+          <t>1577</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>241</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>102</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-14 08:58
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-13 11:43:33</t>
+          <t>取得日時：2026-10-14 08:58:18</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-12</t>
+          <t>比較基準：2026-10-13</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>432</t>
+          <t>435</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>543</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12T22:30:05+0000</t>
+          <t>2026-10-13T22:30:38+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1103,19 +1103,19 @@
           <t>30</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10T13:01:36+0000</t>
+          <t>2026-10-13T12:32:01+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
           <t>28</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1155,9 +1155,9 @@
           <t>68</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1577</t>
+          <t>1578</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1246,12 +1246,12 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1259,24 +1259,24 @@
           <t>348</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12T12:52:38+0000</t>
+          <t>2026-10-13T10:42:29+0000</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1298,32 +1298,32 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>108</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>240</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11T06:05:06+0000</t>
+          <t>2026-10-13T11:15:24+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,19 +1353,19 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>104</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1573,22 +1573,22 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13T12:45:57+0000</t>
+          <t>2026-10-13T16:41:52+0000</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-15 08:29
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-14 09:35:25</t>
+          <t>取得日時：2026-10-15 08:29:12</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-13</t>
+          <t>比較基準：2026-10-14</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>435</t>
+          <t>438</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>544</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13T22:30:38+0000</t>
+          <t>2026-10-14T22:30:05+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>70</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -937,19 +937,19 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>109</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13T12:32:01+0000</t>
+          <t>2026-10-14T12:19:31+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,37 +1142,37 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10T13:52:12+0000</t>
+          <t>2026-10-14T14:52:11+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1578</t>
+          <t>1579</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,9 +1249,9 @@
           <t>59</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1259,7 +1259,7 @@
           <t>348</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1301,9 +1301,9 @@
           <t>108</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,9 +1311,9 @@
           <t>240</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>-1人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1360,12 +1360,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1405,19 +1405,19 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1506,37 +1506,37 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>104</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03T13:08:02+0000</t>
+          <t>2026-10-14T15:57:18+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1563,17 +1563,17 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>182</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-16 08:20
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-15 09:04:37</t>
+          <t>取得日時：2026-10-16 08:20:36</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-14</t>
+          <t>比較基準：2026-10-15</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>441</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>544</t>
+          <t>543</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14T22:30:05+0000</t>
+          <t>2026-10-15T22:35:28+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -726,37 +726,37 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10T15:30:17+0000</t>
+          <t>2026-10-15T08:09:29+0000</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -947,9 +947,9 @@
           <t>110</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14T12:19:31+0000</t>
+          <t>2026-10-15T10:35:01+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>70</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14T14:52:11+0000</t>
+          <t>2026-10-15T14:39:54+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1579</t>
+          <t>1580</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1365,22 +1365,22 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07T02:18:22+0000</t>
+          <t>2026-10-15T23:12:54+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1412,12 +1412,12 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,9 +1509,9 @@
           <t>15</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1519,9 +1519,9 @@
           <t>105</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>182</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-17 08:04
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-16 08:49:26</t>
+          <t>取得日時：2026-10-17 08:04:30</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-15</t>
+          <t>比較基準：2026-10-16</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>441</t>
+          <t>444</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15T22:35:28+0000</t>
+          <t>2026-10-16T22:30:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>79</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+6人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15T10:35:01+0000</t>
+          <t>2026-10-16T10:07:28+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15T14:39:54+0000</t>
+          <t>2026-10-16T10:04:39+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1580</t>
+          <t>1581</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1301,19 +1301,19 @@
           <t>108</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>240</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1355,17 +1355,17 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1405,7 +1405,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1415,9 +1415,9 @@
           <t>54</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>15</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>105</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-10-18 07:42
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-17 08:51:34</t>
+          <t>取得日時：2026-10-18 07:42:59</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-10-16</t>
+          <t>比較基準：2026-10-17</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>447</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16T22:30:06+0000</t>
+          <t>2026-10-17T22:30:04+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>79</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+6人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -937,19 +937,19 @@
           <t>39</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16T10:07:28+0000</t>
+          <t>2026-10-17T12:26:19+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1147,17 +1147,17 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>71</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1581</t>
+          <t>1582</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>109</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1313,22 +1313,22 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13T11:15:24+0000</t>
+          <t>2026-10-17T04:50:05+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>95</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1516,12 +1516,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>